<commit_message>
Fix Total Anggaran calculation + upgrade to professional dashboard
PERBAIKAN PERHITUNGAN:
- Total Anggaran: Rp 3.337.187.500 -> Rp 3.487.166.000 (SUM Dana Alokasi dari 8 Pengaturan)
- Total Penggunaan: Rp 3.198.897.541 (tetap, dari SUM aktual harian)
- Total Sisa Dana: Rp 288.268.459 (bukan 138 jt; nilai sebelumnya salah karena pagu libur=0)
- % Penyerapan: 91.73% (bukan 95.86%)
- Tambahan: % Surplus (Hemat) = 26.12%, % Defisit = 22.15%, Rasio Disiplin = 79.76%

DASHBOARD PROFESIONAL:
- 5 chart: Line (tren harian), Doughnut (komposisi), Pie3D (status), Bar (mingguan), Stacked (alokasi)
- KPI banner 5 kolom dengan ikon & warna
- Border tebal navy pada KPI values
- Section header berwarna per klaster (emerald/orange/purple/emerald)
- Sheet Chart Data terpisah sebagai sumber grafik (mudah di-maintain)
- Catatan metodologi di footer
</commit_message>
<xml_diff>
--- a/Dashboard_Akumulasi_Sep_Des_2025.xlsx
+++ b/Dashboard_Akumulasi_Sep_Des_2025.xlsx
@@ -12,45 +12,46 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="&quot;Rp&quot;\ #,##0;[Red]&quot;Rp&quot;\ \-#,##0"/>
     <numFmt numFmtId="165" formatCode="dd\ mmm\ yyyy"/>
     <numFmt numFmtId="166" formatCode="0.00%"/>
     <numFmt numFmtId="167" formatCode="#,##0"/>
     <numFmt numFmtId="168" formatCode="&quot;Rp&quot;\ #,##0"/>
+    <numFmt numFmtId="169" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="20"/>
+      <sz val="22"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="13"/>
+      <sz val="14"/>
       <color rgb="FF1F3864"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="13"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color rgb="FF1F3864"/>
       <name val="Calibri"/>
     </font>
@@ -85,13 +86,13 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
     </font>
@@ -101,8 +102,32 @@
       <color rgb="FF595959"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1F3864"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF595959"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -169,8 +194,18 @@
         <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF548235"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4B084"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -192,32 +227,46 @@
         <color rgb="FFBFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -226,7 +275,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -246,26 +295,26 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="164" fontId="9" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -273,8 +322,23 @@
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -322,20 +386,12 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:strRef>
-              <c:f>'Chart Data'!$B$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Total Pagu</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:v>Total Pagu</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575">
               <a:solidFill>
-                <a:srgbClr val="70AD47"/>
+                <a:srgbClr val="548235"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -358,15 +414,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:strRef>
-              <c:f>'Chart Data'!$C$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Total Aktual</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:v>Total Aktual</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575">
@@ -448,7 +496,7 @@
     <c:title>
       <c:tx>
         <c:rich>
-          <a:bodyPr/>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
@@ -527,7 +575,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="1">
+                  <a:defRPr sz="1100" b="1">
                     <a:solidFill>
                       <a:srgbClr val="FFFFFF"/>
                     </a:solidFill>
@@ -546,12 +594,12 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Chart Data'!$A$105:$A$107</c:f>
+              <c:f>'Chart Data'!$A$104:$A$106</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Chart Data'!$B$105:$B$107</c:f>
+              <c:f>'Chart Data'!$B$104:$B$106</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -567,11 +615,377 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1000" b="1"/>
+            <a:defRPr sz="1100" b="1"/>
           </a:pPr>
           <a:endParaRPr lang="id-ID"/>
         </a:p>
       </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F3864"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="id-ID" sz="1400" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F3864"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>DISTRIBUSI STATUS HARIAN</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pie3DChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="70AD47"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="A6A6A6"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1100" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="FFFFFF"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="id-ID"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Chart Data'!$A$110:$A$112</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Chart Data'!$B$110:$B$112</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+      </c:pie3DChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1100" b="1"/>
+          </a:pPr>
+          <a:endParaRPr lang="id-ID"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F3864"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="id-ID" sz="1400" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F3864"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>PERBANDINGAN MINGGUAN: Pagu vs Aktual</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Total Pagu</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E75B6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Chart Data'!$A$116:$A$131</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Chart Data'!$B$116:$B$131</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Total Aktual</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="ED7D31"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="843C0C"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Chart Data'!$A$116:$A$131</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Chart Data'!$C$116:$C$131</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="100"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="out"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F3864"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="id-ID" sz="1400" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F3864"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>ALOKASI vs PENGGUNAAN: Pangan &amp; Operasional</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Terpakai</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="ED7D31"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Chart Data'!$A$135:$A$136</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Chart Data'!$C$135:$C$136</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Sisa</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="70AD47"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Chart Data'!$A$135:$A$136</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Chart Data'!$D$135:$D$136</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:overlap val="100"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorTickMark val="out"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
@@ -585,18 +999,18 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>61</xdr:row>
+      <xdr:row>59</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>80</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Line Chart"/>
+        <xdr:cNvPr id="2" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -619,14 +1033,14 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>100</xdr:row>
+      <xdr:row>102</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Doughnut Chart"/>
+        <xdr:cNvPr id="3" name="Chart 2"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -641,6 +1055,96 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>124</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>125</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>142</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -649,16 +1153,18 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">DASHBOARD AKUMULASI LAPORAN KEUANGAN</t>
@@ -671,11 +1177,13 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPPG BATTUWINANGUN - Program Pemenuhan Gizi</t>
+          <t xml:space="preserve">SPPG BATTUWINANGUN  -  Program Pemenuhan Gizi Nasional</t>
         </is>
       </c>
       <c r="B2" s="1"/>
@@ -685,85 +1193,109 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Periode:</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+          <t xml:space="preserve">PERIODE LAPORAN:</t>
+        </is>
+      </c>
+      <c r="B3" s="0"/>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">01 September 2025 s/d 31 Desember 2025</t>
         </is>
       </c>
-      <c r="C3" s="0"/>
       <c r="D3" s="0"/>
       <c r="E3" s="0"/>
       <c r="F3" s="0"/>
-      <c r="G3" s="0"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HARI TERCATAT:</t>
+        </is>
+      </c>
       <c r="H3" s="0"/>
-    </row>
-    <row r="5" ht="22" customHeight="1">
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">97 hari (84 hari aktif)</t>
+        </is>
+      </c>
+      <c r="J3" s="0"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TOTAL DANA ANGGARAN</t>
+          <t xml:space="preserve">💰 TOTAL DANA ANGGARAN</t>
         </is>
       </c>
       <c r="B5" s="0"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TOTAL DIPAKAI</t>
+          <t xml:space="preserve">📊 TOTAL DIPAKAI</t>
         </is>
       </c>
       <c r="D5" s="0"/>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TOTAL SISA DANA</t>
-        </is>
-      </c>
-      <c r="F5" s="0"/>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">% PENYERAPAN</t>
-        </is>
-      </c>
-      <c r="H5" s="0"/>
-    </row>
-    <row r="6" ht="40" customHeight="1">
+      <c r="E5" s="0"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">💵 TOTAL SISA DANA</t>
+        </is>
+      </c>
+      <c r="G5" s="0"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">📈 % PENYERAPAN</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⭐ % SURPLUS (HEMAT)</t>
+        </is>
+      </c>
+      <c r="J5" s="0"/>
+    </row>
+    <row r="6" ht="46" customHeight="1">
       <c r="A6" s="5">
-        <v>3337187500.0</v>
+        <v>3487166000.0</v>
       </c>
       <c r="B6" s="0"/>
       <c r="C6" s="5">
         <v>3198897541.0</v>
       </c>
       <c r="D6" s="0"/>
-      <c r="E6" s="17">
-        <v>138289959.0</v>
-      </c>
-      <c r="F6" s="0"/>
-      <c r="G6" s="8">
-        <v>0.9585609262290476</v>
-      </c>
-      <c r="H6" s="0"/>
-    </row>
-    <row r="8" ht="24" customHeight="1">
+      <c r="E6" s="0"/>
+      <c r="F6" s="17">
+        <v>288268459.0</v>
+      </c>
+      <c r="G6" s="0"/>
+      <c r="H6" s="30">
+        <v>0.9173344604185748</v>
+      </c>
+      <c r="I6" s="30">
+        <v>0.26117636499094105</v>
+      </c>
+      <c r="J6" s="0"/>
+    </row>
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">A. PENGELUARAN BAHAN PANGAN</t>
         </is>
       </c>
-      <c r="B8" s="0"/>
-      <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
-      <c r="E8" s="0"/>
-      <c r="F8" s="0"/>
-      <c r="G8" s="0"/>
-      <c r="H8" s="0"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Rata-Rata Pengeluaran Bahan Pangan / Hari</t>
         </is>
@@ -772,14 +1304,16 @@
       <c r="C9" s="0"/>
       <c r="D9" s="0"/>
       <c r="E9" s="0"/>
-      <c r="F9" s="6">
+      <c r="F9" s="0"/>
+      <c r="G9" s="6">
         <v>24819617.035714287</v>
       </c>
-      <c r="G9" s="0"/>
       <c r="H9" s="0"/>
+      <c r="I9" s="0"/>
+      <c r="J9" s="0"/>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Pengeluaran Bahan Pangan Seharusnya (Pagu) / Hari</t>
         </is>
@@ -788,14 +1322,16 @@
       <c r="C10" s="0"/>
       <c r="D10" s="0"/>
       <c r="E10" s="0"/>
-      <c r="F10" s="6">
+      <c r="F10" s="0"/>
+      <c r="G10" s="6">
         <v>26737047.61904762</v>
       </c>
-      <c r="G10" s="0"/>
       <c r="H10" s="0"/>
+      <c r="I10" s="0"/>
+      <c r="J10" s="0"/>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Selisih Pengeluaran Bahan Pangan / Hari</t>
         </is>
@@ -804,11 +1340,13 @@
       <c r="C11" s="0"/>
       <c r="D11" s="0"/>
       <c r="E11" s="0"/>
-      <c r="F11" s="6">
+      <c r="F11" s="0"/>
+      <c r="G11" s="6">
         <v>1917430.583333332</v>
       </c>
-      <c r="G11" s="0"/>
       <c r="H11" s="0"/>
+      <c r="I11" s="0"/>
+      <c r="J11" s="0"/>
     </row>
     <row r="12">
       <c r="A12" s="0"/>
@@ -819,9 +1357,11 @@
       <c r="F12" s="0"/>
       <c r="G12" s="0"/>
       <c r="H12" s="0"/>
+      <c r="I12" s="0"/>
+      <c r="J12" s="0"/>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Dana Total Bahan Pangan</t>
         </is>
@@ -830,14 +1370,16 @@
       <c r="C13" s="0"/>
       <c r="D13" s="0"/>
       <c r="E13" s="0"/>
-      <c r="F13" s="7">
-        <v>2245912000.0</v>
-      </c>
-      <c r="G13" s="0"/>
+      <c r="F13" s="0"/>
+      <c r="G13" s="7">
+        <v>2276180000.0</v>
+      </c>
       <c r="H13" s="0"/>
+      <c r="I13" s="0"/>
+      <c r="J13" s="0"/>
     </row>
     <row r="14">
-      <c r="A14" s="26" t="inlineStr">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Penggunaan Dana Pangan</t>
         </is>
@@ -846,14 +1388,16 @@
       <c r="C14" s="0"/>
       <c r="D14" s="0"/>
       <c r="E14" s="0"/>
-      <c r="F14" s="7">
+      <c r="F14" s="0"/>
+      <c r="G14" s="7">
         <v>2084847831.0</v>
       </c>
-      <c r="G14" s="0"/>
       <c r="H14" s="0"/>
+      <c r="I14" s="0"/>
+      <c r="J14" s="0"/>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="inlineStr">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Sisa Dana Pangan</t>
         </is>
@@ -862,14 +1406,16 @@
       <c r="C15" s="0"/>
       <c r="D15" s="0"/>
       <c r="E15" s="0"/>
-      <c r="F15" s="7">
-        <v>161064169.0</v>
-      </c>
-      <c r="G15" s="0"/>
+      <c r="F15" s="0"/>
+      <c r="G15" s="7">
+        <v>191332169.0</v>
+      </c>
       <c r="H15" s="0"/>
+      <c r="I15" s="0"/>
+      <c r="J15" s="0"/>
     </row>
     <row r="16">
-      <c r="A16" s="26" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">% Penggunaan Dana Pangan</t>
         </is>
@@ -878,28 +1424,32 @@
       <c r="C16" s="0"/>
       <c r="D16" s="0"/>
       <c r="E16" s="0"/>
-      <c r="F16" s="8">
-        <v>0.9282856278429431</v>
-      </c>
-      <c r="G16" s="0"/>
+      <c r="F16" s="0"/>
+      <c r="G16" s="8">
+        <v>0.9159415472414308</v>
+      </c>
       <c r="H16" s="0"/>
-    </row>
-    <row r="18" ht="24" customHeight="1">
+      <c r="I16" s="0"/>
+      <c r="J16" s="0"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">B. PENGELUARAN OPERASIONAL</t>
         </is>
       </c>
-      <c r="B18" s="0"/>
-      <c r="C18" s="0"/>
-      <c r="D18" s="0"/>
-      <c r="E18" s="0"/>
-      <c r="F18" s="0"/>
-      <c r="G18" s="0"/>
-      <c r="H18" s="0"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
     </row>
     <row r="19">
-      <c r="A19" s="26" t="inlineStr">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Rata-Rata Pengeluaran Operasional / Hari</t>
         </is>
@@ -908,14 +1458,16 @@
       <c r="C19" s="0"/>
       <c r="D19" s="0"/>
       <c r="E19" s="0"/>
-      <c r="F19" s="6">
+      <c r="F19" s="0"/>
+      <c r="G19" s="6">
         <v>13262496.547619049</v>
       </c>
-      <c r="G19" s="0"/>
       <c r="H19" s="0"/>
+      <c r="I19" s="0"/>
+      <c r="J19" s="0"/>
     </row>
     <row r="20">
-      <c r="A20" s="26" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Pengeluaran Operasional Seharusnya (Pagu) / Hari</t>
         </is>
@@ -924,14 +1476,16 @@
       <c r="C20" s="0"/>
       <c r="D20" s="0"/>
       <c r="E20" s="0"/>
-      <c r="F20" s="6">
+      <c r="F20" s="0"/>
+      <c r="G20" s="6">
         <v>12991375.0</v>
       </c>
-      <c r="G20" s="0"/>
       <c r="H20" s="0"/>
+      <c r="I20" s="0"/>
+      <c r="J20" s="0"/>
     </row>
     <row r="21">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Selisih Pengeluaran Operasional / Hari</t>
         </is>
@@ -940,11 +1494,13 @@
       <c r="C21" s="0"/>
       <c r="D21" s="0"/>
       <c r="E21" s="0"/>
-      <c r="F21" s="6">
+      <c r="F21" s="0"/>
+      <c r="G21" s="6">
         <v>-271121.5476190485</v>
       </c>
-      <c r="G21" s="0"/>
       <c r="H21" s="0"/>
+      <c r="I21" s="0"/>
+      <c r="J21" s="0"/>
     </row>
     <row r="22">
       <c r="A22" s="0"/>
@@ -955,9 +1511,11 @@
       <c r="F22" s="0"/>
       <c r="G22" s="0"/>
       <c r="H22" s="0"/>
+      <c r="I22" s="0"/>
+      <c r="J22" s="0"/>
     </row>
     <row r="23">
-      <c r="A23" s="26" t="inlineStr">
+      <c r="A23" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Dana Total Operasional</t>
         </is>
@@ -966,14 +1524,16 @@
       <c r="C23" s="0"/>
       <c r="D23" s="0"/>
       <c r="E23" s="0"/>
-      <c r="F23" s="7">
-        <v>1091275500.0</v>
-      </c>
-      <c r="G23" s="0"/>
+      <c r="F23" s="0"/>
+      <c r="G23" s="7">
+        <v>1210986000.0</v>
+      </c>
       <c r="H23" s="0"/>
+      <c r="I23" s="0"/>
+      <c r="J23" s="0"/>
     </row>
     <row r="24">
-      <c r="A24" s="26" t="inlineStr">
+      <c r="A24" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Penggunaan Dana Operasional</t>
         </is>
@@ -982,14 +1542,16 @@
       <c r="C24" s="0"/>
       <c r="D24" s="0"/>
       <c r="E24" s="0"/>
-      <c r="F24" s="7">
+      <c r="F24" s="0"/>
+      <c r="G24" s="7">
         <v>1114049710.0</v>
       </c>
-      <c r="G24" s="0"/>
       <c r="H24" s="0"/>
+      <c r="I24" s="0"/>
+      <c r="J24" s="0"/>
     </row>
     <row r="25">
-      <c r="A25" s="26" t="inlineStr">
+      <c r="A25" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Sisa Dana Operasional</t>
         </is>
@@ -998,14 +1560,16 @@
       <c r="C25" s="0"/>
       <c r="D25" s="0"/>
       <c r="E25" s="0"/>
-      <c r="F25" s="7">
-        <v>-22774210.0</v>
-      </c>
-      <c r="G25" s="0"/>
+      <c r="F25" s="0"/>
+      <c r="G25" s="7">
+        <v>96936290.0</v>
+      </c>
       <c r="H25" s="0"/>
+      <c r="I25" s="0"/>
+      <c r="J25" s="0"/>
     </row>
     <row r="26">
-      <c r="A26" s="26" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">% Penggunaan Dana Operasional</t>
         </is>
@@ -1014,28 +1578,32 @@
       <c r="C26" s="0"/>
       <c r="D26" s="0"/>
       <c r="E26" s="0"/>
-      <c r="F26" s="8">
-        <v>1.020869349673845</v>
-      </c>
-      <c r="G26" s="0"/>
+      <c r="F26" s="0"/>
+      <c r="G26" s="8">
+        <v>0.9199525923503657</v>
+      </c>
       <c r="H26" s="0"/>
-    </row>
-    <row r="28" ht="24" customHeight="1">
+      <c r="I26" s="0"/>
+      <c r="J26" s="0"/>
+    </row>
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">C. RINGKASAN TOTAL</t>
         </is>
       </c>
-      <c r="B28" s="0"/>
-      <c r="C28" s="0"/>
-      <c r="D28" s="0"/>
-      <c r="E28" s="0"/>
-      <c r="F28" s="0"/>
-      <c r="G28" s="0"/>
-      <c r="H28" s="0"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="25"/>
     </row>
     <row r="29">
-      <c r="A29" s="26" t="inlineStr">
+      <c r="A29" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Dana Anggaran</t>
         </is>
@@ -1044,14 +1612,16 @@
       <c r="C29" s="0"/>
       <c r="D29" s="0"/>
       <c r="E29" s="0"/>
-      <c r="F29" s="7">
-        <v>3337187500.0</v>
-      </c>
-      <c r="G29" s="0"/>
+      <c r="F29" s="0"/>
+      <c r="G29" s="7">
+        <v>3487166000.0</v>
+      </c>
       <c r="H29" s="0"/>
+      <c r="I29" s="0"/>
+      <c r="J29" s="0"/>
     </row>
     <row r="30">
-      <c r="A30" s="26" t="inlineStr">
+      <c r="A30" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Penggunaan Dana</t>
         </is>
@@ -1060,14 +1630,16 @@
       <c r="C30" s="0"/>
       <c r="D30" s="0"/>
       <c r="E30" s="0"/>
-      <c r="F30" s="7">
+      <c r="F30" s="0"/>
+      <c r="G30" s="7">
         <v>3198897541.0</v>
       </c>
-      <c r="G30" s="0"/>
       <c r="H30" s="0"/>
+      <c r="I30" s="0"/>
+      <c r="J30" s="0"/>
     </row>
     <row r="31">
-      <c r="A31" s="26" t="inlineStr">
+      <c r="A31" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Sisa Dana</t>
         </is>
@@ -1076,14 +1648,16 @@
       <c r="C31" s="0"/>
       <c r="D31" s="0"/>
       <c r="E31" s="0"/>
-      <c r="F31" s="7">
-        <v>138289959.0</v>
-      </c>
-      <c r="G31" s="0"/>
+      <c r="F31" s="0"/>
+      <c r="G31" s="7">
+        <v>288268459.0</v>
+      </c>
       <c r="H31" s="0"/>
+      <c r="I31" s="0"/>
+      <c r="J31" s="0"/>
     </row>
     <row r="32">
-      <c r="A32" s="26" t="inlineStr">
+      <c r="A32" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">% Penyerapan Anggaran</t>
         </is>
@@ -1092,11 +1666,13 @@
       <c r="C32" s="0"/>
       <c r="D32" s="0"/>
       <c r="E32" s="0"/>
-      <c r="F32" s="8">
-        <v>0.9585609262290476</v>
-      </c>
-      <c r="G32" s="0"/>
+      <c r="F32" s="0"/>
+      <c r="G32" s="8">
+        <v>0.9173344604185748</v>
+      </c>
       <c r="H32" s="0"/>
+      <c r="I32" s="0"/>
+      <c r="J32" s="0"/>
     </row>
     <row r="33">
       <c r="A33" s="0"/>
@@ -1107,9 +1683,11 @@
       <c r="F33" s="0"/>
       <c r="G33" s="0"/>
       <c r="H33" s="0"/>
+      <c r="I33" s="0"/>
+      <c r="J33" s="0"/>
     </row>
     <row r="34">
-      <c r="A34" s="26" t="inlineStr">
+      <c r="A34" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Rata-Rata Total Pengeluaran / Hari</t>
         </is>
@@ -1118,14 +1696,16 @@
       <c r="C34" s="0"/>
       <c r="D34" s="0"/>
       <c r="E34" s="0"/>
-      <c r="F34" s="6">
+      <c r="F34" s="0"/>
+      <c r="G34" s="6">
         <v>38082113.583333336</v>
       </c>
-      <c r="G34" s="0"/>
       <c r="H34" s="0"/>
+      <c r="I34" s="0"/>
+      <c r="J34" s="0"/>
     </row>
     <row r="35">
-      <c r="A35" s="26" t="inlineStr">
+      <c r="A35" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Pagu Total / Hari (Seharusnya)</t>
         </is>
@@ -1134,14 +1714,16 @@
       <c r="C35" s="0"/>
       <c r="D35" s="0"/>
       <c r="E35" s="0"/>
-      <c r="F35" s="6">
+      <c r="F35" s="0"/>
+      <c r="G35" s="6">
         <v>39728422.61904762</v>
       </c>
-      <c r="G35" s="0"/>
       <c r="H35" s="0"/>
+      <c r="I35" s="0"/>
+      <c r="J35" s="0"/>
     </row>
     <row r="36">
-      <c r="A36" s="26" t="inlineStr">
+      <c r="A36" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Selisih Total / Hari</t>
         </is>
@@ -1150,28 +1732,32 @@
       <c r="C36" s="0"/>
       <c r="D36" s="0"/>
       <c r="E36" s="0"/>
-      <c r="F36" s="6">
+      <c r="F36" s="0"/>
+      <c r="G36" s="6">
         <v>1646309.0357142836</v>
       </c>
-      <c r="G36" s="0"/>
       <c r="H36" s="0"/>
-    </row>
-    <row r="38" ht="24" customHeight="1">
+      <c r="I36" s="0"/>
+      <c r="J36" s="0"/>
+    </row>
+    <row r="38" ht="28" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">D. ANALISIS SURPLUS / DEFISIT</t>
         </is>
       </c>
-      <c r="B38" s="0"/>
-      <c r="C38" s="0"/>
-      <c r="D38" s="0"/>
-      <c r="E38" s="0"/>
-      <c r="F38" s="0"/>
-      <c r="G38" s="0"/>
-      <c r="H38" s="0"/>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
     </row>
     <row r="39">
-      <c r="A39" s="26" t="inlineStr">
+      <c r="A39" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Jumlah Hari SURPLUS (Pengeluaran &lt; Pagu)</t>
         </is>
@@ -1180,14 +1766,16 @@
       <c r="C39" s="0"/>
       <c r="D39" s="0"/>
       <c r="E39" s="0"/>
-      <c r="F39" s="20">
+      <c r="F39" s="0"/>
+      <c r="G39" s="20">
         <v>67</v>
       </c>
-      <c r="G39" s="0"/>
       <c r="H39" s="0"/>
+      <c r="I39" s="0"/>
+      <c r="J39" s="0"/>
     </row>
     <row r="40">
-      <c r="A40" s="26" t="inlineStr">
+      <c r="A40" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Jumlah Hari DEFISIT (Pengeluaran &gt; Pagu)</t>
         </is>
@@ -1196,30 +1784,34 @@
       <c r="C40" s="0"/>
       <c r="D40" s="0"/>
       <c r="E40" s="0"/>
-      <c r="F40" s="20">
+      <c r="F40" s="0"/>
+      <c r="G40" s="20">
         <v>17</v>
       </c>
-      <c r="G40" s="0"/>
       <c r="H40" s="0"/>
+      <c r="I40" s="0"/>
+      <c r="J40" s="0"/>
     </row>
     <row r="41">
-      <c r="A41" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jumlah Hari AMAN (Pengeluaran = Pagu / Libur)</t>
+      <c r="A41" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jumlah Hari AMAN (Libur / Pas Pagu)</t>
         </is>
       </c>
       <c r="B41" s="0"/>
       <c r="C41" s="0"/>
       <c r="D41" s="0"/>
       <c r="E41" s="0"/>
-      <c r="F41" s="20">
+      <c r="F41" s="0"/>
+      <c r="G41" s="20">
         <v>13</v>
       </c>
-      <c r="G41" s="0"/>
       <c r="H41" s="0"/>
+      <c r="I41" s="0"/>
+      <c r="J41" s="0"/>
     </row>
     <row r="42">
-      <c r="A42" s="26" t="inlineStr">
+      <c r="A42" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Jumlah Hari Belum Input</t>
         </is>
@@ -1228,11 +1820,13 @@
       <c r="C42" s="0"/>
       <c r="D42" s="0"/>
       <c r="E42" s="0"/>
-      <c r="F42" s="20">
+      <c r="F42" s="0"/>
+      <c r="G42" s="20">
         <v>0</v>
       </c>
-      <c r="G42" s="0"/>
       <c r="H42" s="0"/>
+      <c r="I42" s="0"/>
+      <c r="J42" s="0"/>
     </row>
     <row r="43">
       <c r="A43" s="0"/>
@@ -1243,9 +1837,11 @@
       <c r="F43" s="0"/>
       <c r="G43" s="0"/>
       <c r="H43" s="0"/>
+      <c r="I43" s="0"/>
+      <c r="J43" s="0"/>
     </row>
     <row r="44">
-      <c r="A44" s="26" t="inlineStr">
+      <c r="A44" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Akumulasi Surplus</t>
         </is>
@@ -1254,14 +1850,16 @@
       <c r="C44" s="0"/>
       <c r="D44" s="0"/>
       <c r="E44" s="0"/>
-      <c r="F44" s="22">
+      <c r="F44" s="0"/>
+      <c r="G44" s="22">
         <v>910765340.0</v>
       </c>
-      <c r="G44" s="0"/>
       <c r="H44" s="0"/>
+      <c r="I44" s="0"/>
+      <c r="J44" s="0"/>
     </row>
     <row r="45">
-      <c r="A45" s="26" t="inlineStr">
+      <c r="A45" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Akumulasi Defisit</t>
         </is>
@@ -1270,14 +1868,16 @@
       <c r="C45" s="0"/>
       <c r="D45" s="0"/>
       <c r="E45" s="0"/>
-      <c r="F45" s="23">
+      <c r="F45" s="0"/>
+      <c r="G45" s="23">
         <v>-772475381.0</v>
       </c>
-      <c r="G45" s="0"/>
       <c r="H45" s="0"/>
+      <c r="I45" s="0"/>
+      <c r="J45" s="0"/>
     </row>
     <row r="46">
-      <c r="A46" s="26" t="inlineStr">
+      <c r="A46" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Net Surplus / Defisit</t>
         </is>
@@ -1286,260 +1886,397 @@
       <c r="C46" s="0"/>
       <c r="D46" s="0"/>
       <c r="E46" s="0"/>
-      <c r="F46" s="7">
+      <c r="F46" s="0"/>
+      <c r="G46" s="7">
         <v>138289959.0</v>
       </c>
-      <c r="G46" s="0"/>
       <c r="H46" s="0"/>
+      <c r="I46" s="0"/>
+      <c r="J46" s="0"/>
     </row>
     <row r="47">
-      <c r="A47" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">% Surplus Total (dari Total Pagu)</t>
+      <c r="A47" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% Surplus dari Total Anggaran</t>
         </is>
       </c>
       <c r="B47" s="0"/>
       <c r="C47" s="0"/>
       <c r="D47" s="0"/>
       <c r="E47" s="0"/>
-      <c r="F47" s="8">
-        <v>0.04143907377095234</v>
-      </c>
-      <c r="G47" s="0"/>
+      <c r="F47" s="0"/>
+      <c r="G47" s="30">
+        <v>0.26117636499094105</v>
+      </c>
       <c r="H47" s="0"/>
+      <c r="I47" s="0"/>
+      <c r="J47" s="0"/>
     </row>
     <row r="48">
-      <c r="A48" s="0"/>
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% Defisit dari Total Anggaran</t>
+        </is>
+      </c>
       <c r="B48" s="0"/>
       <c r="C48" s="0"/>
       <c r="D48" s="0"/>
       <c r="E48" s="0"/>
       <c r="F48" s="0"/>
-      <c r="G48" s="0"/>
+      <c r="G48" s="31">
+        <v>0.22151953219319068</v>
+      </c>
       <c r="H48" s="0"/>
+      <c r="I48" s="0"/>
+      <c r="J48" s="0"/>
     </row>
     <row r="49">
-      <c r="A49" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pengeluaran Tertinggi / Hari (Rp)</t>
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rasio Disiplin Anggaran (Hari Surplus / Aktif Non-Libur)</t>
         </is>
       </c>
       <c r="B49" s="0"/>
       <c r="C49" s="0"/>
       <c r="D49" s="0"/>
       <c r="E49" s="0"/>
-      <c r="F49" s="7">
-        <v>132539500.0</v>
-      </c>
-      <c r="G49" s="0"/>
+      <c r="F49" s="0"/>
+      <c r="G49" s="8">
+        <v>0.7976190476190477</v>
+      </c>
       <c r="H49" s="0"/>
+      <c r="I49" s="0"/>
+      <c r="J49" s="0"/>
     </row>
     <row r="50">
-      <c r="A50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Tanggal Pengeluaran Tertinggi</t>
-        </is>
-      </c>
+      <c r="A50" s="0"/>
       <c r="B50" s="0"/>
       <c r="C50" s="0"/>
       <c r="D50" s="0"/>
       <c r="E50" s="0"/>
-      <c r="F50" s="16">
-        <v>45983</v>
-      </c>
+      <c r="F50" s="0"/>
       <c r="G50" s="0"/>
       <c r="H50" s="0"/>
+      <c r="I50" s="0"/>
+      <c r="J50" s="0"/>
     </row>
     <row r="51">
-      <c r="A51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pengeluaran Terendah / Hari (Rp)</t>
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pengeluaran Tertinggi / Hari (Rp)</t>
         </is>
       </c>
       <c r="B51" s="0"/>
       <c r="C51" s="0"/>
       <c r="D51" s="0"/>
       <c r="E51" s="0"/>
-      <c r="F51" s="7">
-        <v>351800.0</v>
-      </c>
-      <c r="G51" s="0"/>
+      <c r="F51" s="0"/>
+      <c r="G51" s="23">
+        <v>132539500.0</v>
+      </c>
       <c r="H51" s="0"/>
+      <c r="I51" s="0"/>
+      <c r="J51" s="0"/>
     </row>
     <row r="52">
-      <c r="A52" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Tanggal Pengeluaran Terendah</t>
+      <c r="A52" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Tanggal Pengeluaran Tertinggi</t>
         </is>
       </c>
       <c r="B52" s="0"/>
       <c r="C52" s="0"/>
       <c r="D52" s="0"/>
       <c r="E52" s="0"/>
-      <c r="F52" s="16">
+      <c r="F52" s="0"/>
+      <c r="G52" s="16">
+        <v>45983</v>
+      </c>
+      <c r="H52" s="0"/>
+      <c r="I52" s="0"/>
+      <c r="J52" s="0"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pengeluaran Terendah / Hari (Rp)</t>
+        </is>
+      </c>
+      <c r="B53" s="0"/>
+      <c r="C53" s="0"/>
+      <c r="D53" s="0"/>
+      <c r="E53" s="0"/>
+      <c r="F53" s="0"/>
+      <c r="G53" s="22">
+        <v>351800.0</v>
+      </c>
+      <c r="H53" s="0"/>
+      <c r="I53" s="0"/>
+      <c r="J53" s="0"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Tanggal Pengeluaran Terendah</t>
+        </is>
+      </c>
+      <c r="B54" s="0"/>
+      <c r="C54" s="0"/>
+      <c r="D54" s="0"/>
+      <c r="E54" s="0"/>
+      <c r="F54" s="0"/>
+      <c r="G54" s="16">
         <v>46018</v>
       </c>
-      <c r="G52" s="0"/>
-      <c r="H52" s="0"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CATATAN:</t>
-        </is>
-      </c>
-      <c r="B55" s="0"/>
-      <c r="C55" s="0"/>
-      <c r="D55" s="0"/>
-      <c r="E55" s="0"/>
-      <c r="F55" s="0"/>
-      <c r="G55" s="0"/>
-      <c r="H55" s="0"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">- Dashboard akumulatif seluruh periode 01 Sep s/d 31 Des 2025 (97 hari, 84 hari aktif).</t>
-        </is>
-      </c>
-      <c r="B56" s="0"/>
-      <c r="C56" s="0"/>
-      <c r="D56" s="0"/>
-      <c r="E56" s="0"/>
-      <c r="F56" s="0"/>
-      <c r="G56" s="0"/>
-      <c r="H56" s="0"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">- Semua nilai Rupiah sudah divalidasi silang (Pagu - Penggunaan = Sisa = Net Surplus/Defisit).</t>
-        </is>
-      </c>
-      <c r="B57" s="0"/>
-      <c r="C57" s="0"/>
-      <c r="D57" s="0"/>
-      <c r="E57" s="0"/>
-      <c r="F57" s="0"/>
-      <c r="G57" s="0"/>
-      <c r="H57" s="0"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">- Selisih POSITIF = HEMAT (surplus). Selisih NEGATIF = BOROS (defisit).</t>
-        </is>
-      </c>
-      <c r="B58" s="0"/>
-      <c r="C58" s="0"/>
-      <c r="D58" s="0"/>
-      <c r="E58" s="0"/>
-      <c r="F58" s="0"/>
-      <c r="G58" s="0"/>
-      <c r="H58" s="0"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">- Sumber data: 8 file 'Total Akumulasi *.xlsx' di repository.</t>
-        </is>
-      </c>
-      <c r="B59" s="0"/>
-      <c r="C59" s="0"/>
-      <c r="D59" s="0"/>
-      <c r="E59" s="0"/>
-      <c r="F59" s="0"/>
-      <c r="G59" s="0"/>
-      <c r="H59" s="0"/>
+      <c r="H54" s="0"/>
+      <c r="I54" s="0"/>
+      <c r="J54" s="0"/>
+    </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">📊 VISUALISASI GRAFIK EKSEKUTIF</t>
+        </is>
+      </c>
+      <c r="B58" s="3"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+      <c r="I58" s="3"/>
+      <c r="J58" s="3"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CATATAN &amp; METODOLOGI:</t>
+        </is>
+      </c>
+      <c r="B144" s="0"/>
+      <c r="C144" s="0"/>
+      <c r="D144" s="0"/>
+      <c r="E144" s="0"/>
+      <c r="F144" s="0"/>
+      <c r="G144" s="0"/>
+      <c r="H144" s="0"/>
+      <c r="I144" s="0"/>
+      <c r="J144" s="0"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Total Anggaran Rp 3,487,166,000 = SUM Dana Alokasi dari 8 file periode (sheet Pengaturan).</t>
+        </is>
+      </c>
+      <c r="B145" s="0"/>
+      <c r="C145" s="0"/>
+      <c r="D145" s="0"/>
+      <c r="E145" s="0"/>
+      <c r="F145" s="0"/>
+      <c r="G145" s="0"/>
+      <c r="H145" s="0"/>
+      <c r="I145" s="0"/>
+      <c r="J145" s="0"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Total Penggunaan = SUM aktual harian Pangan + Operasional (97 hari tercatat).</t>
+        </is>
+      </c>
+      <c r="B146" s="0"/>
+      <c r="C146" s="0"/>
+      <c r="D146" s="0"/>
+      <c r="E146" s="0"/>
+      <c r="F146" s="0"/>
+      <c r="G146" s="0"/>
+      <c r="H146" s="0"/>
+      <c r="I146" s="0"/>
+      <c r="J146" s="0"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• VALIDASI SILANG: Total Anggaran − Total Penggunaan = Total Sisa = Rp 288.268.459 ✓</t>
+        </is>
+      </c>
+      <c r="B147" s="0"/>
+      <c r="C147" s="0"/>
+      <c r="D147" s="0"/>
+      <c r="E147" s="0"/>
+      <c r="F147" s="0"/>
+      <c r="G147" s="0"/>
+      <c r="H147" s="0"/>
+      <c r="I147" s="0"/>
+      <c r="J147" s="0"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• % Penyerapan = Total Penggunaan / Total Anggaran.</t>
+        </is>
+      </c>
+      <c r="B148" s="0"/>
+      <c r="C148" s="0"/>
+      <c r="D148" s="0"/>
+      <c r="E148" s="0"/>
+      <c r="F148" s="0"/>
+      <c r="G148" s="0"/>
+      <c r="H148" s="0"/>
+      <c r="I148" s="0"/>
+      <c r="J148" s="0"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• % Surplus = Total Akumulasi Hemat (hari SURPLUS saja) / Total Anggaran.</t>
+        </is>
+      </c>
+      <c r="B149" s="0"/>
+      <c r="C149" s="0"/>
+      <c r="D149" s="0"/>
+      <c r="E149" s="0"/>
+      <c r="F149" s="0"/>
+      <c r="G149" s="0"/>
+      <c r="H149" s="0"/>
+      <c r="I149" s="0"/>
+      <c r="J149" s="0"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Selisih POSITIF = HEMAT (surplus). Selisih NEGATIF = BOROS (defisit).</t>
+        </is>
+      </c>
+      <c r="B150" s="0"/>
+      <c r="C150" s="0"/>
+      <c r="D150" s="0"/>
+      <c r="E150" s="0"/>
+      <c r="F150" s="0"/>
+      <c r="G150" s="0"/>
+      <c r="H150" s="0"/>
+      <c r="I150" s="0"/>
+      <c r="J150" s="0"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Sumber: 8 file 'Total Akumulasi *.xlsx' di repository.</t>
+        </is>
+      </c>
+      <c r="B151" s="0"/>
+      <c r="C151" s="0"/>
+      <c r="D151" s="0"/>
+      <c r="E151" s="0"/>
+      <c r="F151" s="0"/>
+      <c r="G151" s="0"/>
+      <c r="H151" s="0"/>
+      <c r="I151" s="0"/>
+      <c r="J151" s="0"/>
     </row>
   </sheetData>
-  <mergeCells count="86">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B3:H3"/>
+  <mergeCells count="99">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:J5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="G6:H6"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="F10:H10"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="F11:H11"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="A31:E31"/>
-    <mergeCell ref="F31:H31"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="A36:E36"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="F39:H39"/>
-    <mergeCell ref="A40:E40"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="F41:H41"/>
-    <mergeCell ref="A42:E42"/>
-    <mergeCell ref="F42:H42"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="F44:H44"/>
-    <mergeCell ref="A45:E45"/>
-    <mergeCell ref="F45:H45"/>
-    <mergeCell ref="A46:E46"/>
-    <mergeCell ref="F46:H46"/>
-    <mergeCell ref="A47:E47"/>
-    <mergeCell ref="F47:H47"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="F51:H51"/>
-    <mergeCell ref="A52:E52"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="A55:H55"/>
-    <mergeCell ref="A56:H56"/>
-    <mergeCell ref="A57:H57"/>
-    <mergeCell ref="A58:H58"/>
-    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="G9:J9"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="G11:J11"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="G13:J13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="G14:J14"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="G15:J15"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="A28:J28"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="G34:J34"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="G35:J35"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="G36:J36"/>
+    <mergeCell ref="A38:J38"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="G40:J40"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="G41:J41"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="G42:J42"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="G44:J44"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="G45:J45"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="G46:J46"/>
+    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="G47:J47"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="G48:J48"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="G49:J49"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="G51:J51"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="G52:J52"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="G53:J53"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="G54:J54"/>
+    <mergeCell ref="A58:J58"/>
+    <mergeCell ref="A144:J144"/>
+    <mergeCell ref="A145:J145"/>
+    <mergeCell ref="A146:J146"/>
+    <mergeCell ref="A147:J147"/>
+    <mergeCell ref="A148:J148"/>
+    <mergeCell ref="A149:J149"/>
+    <mergeCell ref="A150:J150"/>
+    <mergeCell ref="A151:J151"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -6160,11 +6897,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -6177,6 +6914,7 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
@@ -6192,6 +6930,16 @@
       <c r="C3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Aktual</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pangan Aktual</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operasional Aktual</t>
         </is>
       </c>
     </row>
@@ -6205,6 +6953,12 @@
       <c r="C4" s="10">
         <v>43104300.0</v>
       </c>
+      <c r="D4" s="10">
+        <v>31728300.0</v>
+      </c>
+      <c r="E4" s="10">
+        <v>11376000.0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16">
@@ -6216,6 +6970,12 @@
       <c r="C5" s="10">
         <v>30894700.0</v>
       </c>
+      <c r="D5" s="10">
+        <v>29861200.0</v>
+      </c>
+      <c r="E5" s="10">
+        <v>1033500.0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16">
@@ -6227,6 +6987,12 @@
       <c r="C6" s="10">
         <v>30149000.0</v>
       </c>
+      <c r="D6" s="10">
+        <v>27381000.0</v>
+      </c>
+      <c r="E6" s="10">
+        <v>2768000.0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16">
@@ -6238,6 +7004,12 @@
       <c r="C7" s="10">
         <v>39041000.0</v>
       </c>
+      <c r="D7" s="10">
+        <v>20791000.0</v>
+      </c>
+      <c r="E7" s="10">
+        <v>18250000.0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16">
@@ -6249,6 +7021,12 @@
       <c r="C8" s="10">
         <v>0.0</v>
       </c>
+      <c r="D8" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E8" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16">
@@ -6260,6 +7038,12 @@
       <c r="C9" s="10">
         <v>0.0</v>
       </c>
+      <c r="D9" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E9" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="16">
@@ -6271,6 +7055,12 @@
       <c r="C10" s="10">
         <v>0.0</v>
       </c>
+      <c r="D10" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E10" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16">
@@ -6282,6 +7072,12 @@
       <c r="C11" s="10">
         <v>29469050.0</v>
       </c>
+      <c r="D11" s="10">
+        <v>23935050.0</v>
+      </c>
+      <c r="E11" s="10">
+        <v>5534000.0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="16">
@@ -6293,6 +7089,12 @@
       <c r="C12" s="10">
         <v>22762300.0</v>
       </c>
+      <c r="D12" s="10">
+        <v>22762300.0</v>
+      </c>
+      <c r="E12" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16">
@@ -6304,6 +7106,12 @@
       <c r="C13" s="10">
         <v>17952300.0</v>
       </c>
+      <c r="D13" s="10">
+        <v>16132300.0</v>
+      </c>
+      <c r="E13" s="10">
+        <v>1820000.0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="16">
@@ -6315,6 +7123,12 @@
       <c r="C14" s="10">
         <v>25671100.0</v>
       </c>
+      <c r="D14" s="10">
+        <v>23274600.0</v>
+      </c>
+      <c r="E14" s="10">
+        <v>2396500.0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="16">
@@ -6326,6 +7140,12 @@
       <c r="C15" s="10">
         <v>103026181.0</v>
       </c>
+      <c r="D15" s="10">
+        <v>25527681.0</v>
+      </c>
+      <c r="E15" s="10">
+        <v>77498500.0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="16">
@@ -6337,6 +7157,12 @@
       <c r="C16" s="10">
         <v>22361292.0</v>
       </c>
+      <c r="D16" s="10">
+        <v>18746100.0</v>
+      </c>
+      <c r="E16" s="10">
+        <v>3615192.0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16">
@@ -6348,6 +7174,12 @@
       <c r="C17" s="10">
         <v>26042300.0</v>
       </c>
+      <c r="D17" s="10">
+        <v>24222300.0</v>
+      </c>
+      <c r="E17" s="10">
+        <v>1820000.0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="16">
@@ -6359,6 +7191,12 @@
       <c r="C18" s="10">
         <v>27657600.0</v>
       </c>
+      <c r="D18" s="10">
+        <v>25316100.0</v>
+      </c>
+      <c r="E18" s="10">
+        <v>2341500.0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16">
@@ -6370,6 +7208,12 @@
       <c r="C19" s="10">
         <v>27805600.0</v>
       </c>
+      <c r="D19" s="10">
+        <v>25425600.0</v>
+      </c>
+      <c r="E19" s="10">
+        <v>2380000.0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="16">
@@ -6381,6 +7225,12 @@
       <c r="C20" s="10">
         <v>64708500.0</v>
       </c>
+      <c r="D20" s="10">
+        <v>31681000.0</v>
+      </c>
+      <c r="E20" s="10">
+        <v>33027500.0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="16">
@@ -6392,6 +7242,12 @@
       <c r="C21" s="10">
         <v>0.0</v>
       </c>
+      <c r="D21" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E21" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="16">
@@ -6403,6 +7259,12 @@
       <c r="C22" s="10">
         <v>0.0</v>
       </c>
+      <c r="D22" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E22" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="16">
@@ -6414,6 +7276,12 @@
       <c r="C23" s="10">
         <v>27673600.0</v>
       </c>
+      <c r="D23" s="10">
+        <v>24646600.0</v>
+      </c>
+      <c r="E23" s="10">
+        <v>3027000.0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="16">
@@ -6425,6 +7293,12 @@
       <c r="C24" s="10">
         <v>20987600.0</v>
       </c>
+      <c r="D24" s="10">
+        <v>19167600.0</v>
+      </c>
+      <c r="E24" s="10">
+        <v>1820000.0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="16">
@@ -6436,6 +7310,12 @@
       <c r="C25" s="10">
         <v>25771100.0</v>
       </c>
+      <c r="D25" s="10">
+        <v>23418100.0</v>
+      </c>
+      <c r="E25" s="10">
+        <v>2353000.0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="16">
@@ -6447,6 +7327,12 @@
       <c r="C26" s="10">
         <v>28892700.0</v>
       </c>
+      <c r="D26" s="10">
+        <v>26283100.0</v>
+      </c>
+      <c r="E26" s="10">
+        <v>2609600.0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="16">
@@ -6458,6 +7344,12 @@
       <c r="C27" s="10">
         <v>117835500.0</v>
       </c>
+      <c r="D27" s="10">
+        <v>33137500.0</v>
+      </c>
+      <c r="E27" s="10">
+        <v>84698000.0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="16">
@@ -6469,6 +7361,12 @@
       <c r="C28" s="10">
         <v>31101100.0</v>
       </c>
+      <c r="D28" s="10">
+        <v>29281100.0</v>
+      </c>
+      <c r="E28" s="10">
+        <v>1820000.0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="16">
@@ -6480,6 +7378,12 @@
       <c r="C29" s="10">
         <v>26261850.0</v>
       </c>
+      <c r="D29" s="10">
+        <v>23860600.0</v>
+      </c>
+      <c r="E29" s="10">
+        <v>2401250.0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="16">
@@ -6491,6 +7395,12 @@
       <c r="C30" s="10">
         <v>31588600.0</v>
       </c>
+      <c r="D30" s="10">
+        <v>27561600.0</v>
+      </c>
+      <c r="E30" s="10">
+        <v>4027000.0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="16">
@@ -6502,6 +7412,12 @@
       <c r="C31" s="10">
         <v>24573600.0</v>
       </c>
+      <c r="D31" s="10">
+        <v>22518600.0</v>
+      </c>
+      <c r="E31" s="10">
+        <v>2055000.0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="16">
@@ -6513,6 +7429,12 @@
       <c r="C32" s="10">
         <v>65830100.0</v>
       </c>
+      <c r="D32" s="10">
+        <v>32791100.0</v>
+      </c>
+      <c r="E32" s="10">
+        <v>33039000.0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="16">
@@ -6524,6 +7446,12 @@
       <c r="C33" s="10">
         <v>0.0</v>
       </c>
+      <c r="D33" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E33" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="16">
@@ -6535,6 +7463,12 @@
       <c r="C34" s="10">
         <v>0.0</v>
       </c>
+      <c r="D34" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E34" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="16">
@@ -6546,6 +7480,12 @@
       <c r="C35" s="10">
         <v>28586635.0</v>
       </c>
+      <c r="D35" s="10">
+        <v>26154600.0</v>
+      </c>
+      <c r="E35" s="10">
+        <v>2432035.0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="16">
@@ -6557,6 +7497,12 @@
       <c r="C36" s="10">
         <v>22356687.0</v>
       </c>
+      <c r="D36" s="10">
+        <v>19779100.0</v>
+      </c>
+      <c r="E36" s="10">
+        <v>2577587.0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16">
@@ -6568,6 +7514,12 @@
       <c r="C37" s="10">
         <v>22796600.0</v>
       </c>
+      <c r="D37" s="10">
+        <v>19803100.0</v>
+      </c>
+      <c r="E37" s="10">
+        <v>2993500.0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="16">
@@ -6579,6 +7531,12 @@
       <c r="C38" s="10">
         <v>27932600.0</v>
       </c>
+      <c r="D38" s="10">
+        <v>26052600.0</v>
+      </c>
+      <c r="E38" s="10">
+        <v>1880000.0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="16">
@@ -6590,6 +7548,12 @@
       <c r="C39" s="10">
         <v>119622000.0</v>
       </c>
+      <c r="D39" s="10">
+        <v>33657000.0</v>
+      </c>
+      <c r="E39" s="10">
+        <v>85965000.0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="16">
@@ -6601,6 +7565,12 @@
       <c r="C40" s="10">
         <v>26148600.0</v>
       </c>
+      <c r="D40" s="10">
+        <v>23768600.0</v>
+      </c>
+      <c r="E40" s="10">
+        <v>2380000.0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="16">
@@ -6612,6 +7582,12 @@
       <c r="C41" s="10">
         <v>22249100.0</v>
       </c>
+      <c r="D41" s="10">
+        <v>20329100.0</v>
+      </c>
+      <c r="E41" s="10">
+        <v>1920000.0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="16">
@@ -6623,6 +7599,12 @@
       <c r="C42" s="10">
         <v>27252600.0</v>
       </c>
+      <c r="D42" s="10">
+        <v>22749600.0</v>
+      </c>
+      <c r="E42" s="10">
+        <v>4503000.0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="16">
@@ -6634,6 +7616,12 @@
       <c r="C43" s="10">
         <v>24594600.0</v>
       </c>
+      <c r="D43" s="10">
+        <v>21705600.0</v>
+      </c>
+      <c r="E43" s="10">
+        <v>2889000.0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="16">
@@ -6645,6 +7633,12 @@
       <c r="C44" s="10">
         <v>56336500.0</v>
       </c>
+      <c r="D44" s="10">
+        <v>24057500.0</v>
+      </c>
+      <c r="E44" s="10">
+        <v>32279000.0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="16">
@@ -6656,6 +7650,12 @@
       <c r="C45" s="10">
         <v>0.0</v>
       </c>
+      <c r="D45" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E45" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16">
@@ -6667,6 +7667,12 @@
       <c r="C46" s="10">
         <v>0.0</v>
       </c>
+      <c r="D46" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E46" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="16">
@@ -6678,6 +7684,12 @@
       <c r="C47" s="10">
         <v>26125100.0</v>
       </c>
+      <c r="D47" s="10">
+        <v>23441100.0</v>
+      </c>
+      <c r="E47" s="10">
+        <v>2684000.0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="16">
@@ -6689,6 +7701,12 @@
       <c r="C48" s="10">
         <v>25736700.0</v>
       </c>
+      <c r="D48" s="10">
+        <v>23856700.0</v>
+      </c>
+      <c r="E48" s="10">
+        <v>1880000.0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="16">
@@ -6700,6 +7718,12 @@
       <c r="C49" s="10">
         <v>25679700.0</v>
       </c>
+      <c r="D49" s="10">
+        <v>23634700.0</v>
+      </c>
+      <c r="E49" s="10">
+        <v>2045000.0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="16">
@@ -6711,6 +7735,12 @@
       <c r="C50" s="10">
         <v>38156700.0</v>
       </c>
+      <c r="D50" s="10">
+        <v>35704700.0</v>
+      </c>
+      <c r="E50" s="10">
+        <v>2452000.0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="16">
@@ -6722,6 +7752,12 @@
       <c r="C51" s="10">
         <v>123169800.0</v>
       </c>
+      <c r="D51" s="10">
+        <v>39115800.0</v>
+      </c>
+      <c r="E51" s="10">
+        <v>84054000.0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="16">
@@ -6733,6 +7769,12 @@
       <c r="C52" s="10">
         <v>26096371.0</v>
       </c>
+      <c r="D52" s="10">
+        <v>22893500.0</v>
+      </c>
+      <c r="E52" s="10">
+        <v>3202871.0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="16">
@@ -6744,6 +7786,12 @@
       <c r="C53" s="10">
         <v>26625500.0</v>
       </c>
+      <c r="D53" s="10">
+        <v>24745500.0</v>
+      </c>
+      <c r="E53" s="10">
+        <v>1880000.0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="16">
@@ -6755,6 +7803,12 @@
       <c r="C54" s="10">
         <v>37762500.0</v>
       </c>
+      <c r="D54" s="10">
+        <v>34323500.0</v>
+      </c>
+      <c r="E54" s="10">
+        <v>3439000.0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="16">
@@ -6766,6 +7820,12 @@
       <c r="C55" s="10">
         <v>33312000.0</v>
       </c>
+      <c r="D55" s="10">
+        <v>31432000.0</v>
+      </c>
+      <c r="E55" s="10">
+        <v>1880000.0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="16">
@@ -6777,6 +7837,12 @@
       <c r="C56" s="10">
         <v>28077500.0</v>
       </c>
+      <c r="D56" s="10">
+        <v>24713500.0</v>
+      </c>
+      <c r="E56" s="10">
+        <v>3364000.0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="16">
@@ -6788,6 +7854,12 @@
       <c r="C57" s="10">
         <v>70758500.0</v>
       </c>
+      <c r="D57" s="10">
+        <v>29132500.0</v>
+      </c>
+      <c r="E57" s="10">
+        <v>41626000.0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="16">
@@ -6799,6 +7871,12 @@
       <c r="C58" s="10">
         <v>0.0</v>
       </c>
+      <c r="D58" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E58" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="16">
@@ -6810,6 +7888,12 @@
       <c r="C59" s="10">
         <v>28734000.0</v>
       </c>
+      <c r="D59" s="10">
+        <v>26254000.0</v>
+      </c>
+      <c r="E59" s="10">
+        <v>2480000.0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="16">
@@ -6821,6 +7905,12 @@
       <c r="C60" s="10">
         <v>33337800.0</v>
       </c>
+      <c r="D60" s="10">
+        <v>30084800.0</v>
+      </c>
+      <c r="E60" s="10">
+        <v>3253000.0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="16">
@@ -6832,6 +7922,12 @@
       <c r="C61" s="10">
         <v>31112900.0</v>
       </c>
+      <c r="D61" s="10">
+        <v>28144300.0</v>
+      </c>
+      <c r="E61" s="10">
+        <v>2968600.0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="16">
@@ -6843,6 +7939,12 @@
       <c r="C62" s="10">
         <v>25925000.0</v>
       </c>
+      <c r="D62" s="10">
+        <v>22981000.0</v>
+      </c>
+      <c r="E62" s="10">
+        <v>2944000.0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="16">
@@ -6854,6 +7956,12 @@
       <c r="C63" s="10">
         <v>37839500.0</v>
       </c>
+      <c r="D63" s="10">
+        <v>34830500.0</v>
+      </c>
+      <c r="E63" s="10">
+        <v>3009000.0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="16">
@@ -6865,6 +7973,12 @@
       <c r="C64" s="10">
         <v>131157000.0</v>
       </c>
+      <c r="D64" s="10">
+        <v>23784000.0</v>
+      </c>
+      <c r="E64" s="10">
+        <v>107373000.0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="16">
@@ -6876,6 +7990,12 @@
       <c r="C65" s="10">
         <v>32357000.0</v>
       </c>
+      <c r="D65" s="10">
+        <v>29757000.0</v>
+      </c>
+      <c r="E65" s="10">
+        <v>2600000.0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="16">
@@ -6887,6 +8007,12 @@
       <c r="C66" s="10">
         <v>39368300.0</v>
       </c>
+      <c r="D66" s="10">
+        <v>34716300.0</v>
+      </c>
+      <c r="E66" s="10">
+        <v>4652000.0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="16">
@@ -6898,6 +8024,12 @@
       <c r="C67" s="10">
         <v>28285800.0</v>
       </c>
+      <c r="D67" s="10">
+        <v>26047800.0</v>
+      </c>
+      <c r="E67" s="10">
+        <v>2238000.0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="16">
@@ -6909,6 +8041,12 @@
       <c r="C68" s="10">
         <v>30320000.0</v>
       </c>
+      <c r="D68" s="10">
+        <v>26520000.0</v>
+      </c>
+      <c r="E68" s="10">
+        <v>3800000.0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="16">
@@ -6920,6 +8058,12 @@
       <c r="C69" s="10">
         <v>44172000.0</v>
       </c>
+      <c r="D69" s="10">
+        <v>40582500.0</v>
+      </c>
+      <c r="E69" s="10">
+        <v>3589500.0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="16">
@@ -6931,6 +8075,12 @@
       <c r="C70" s="10">
         <v>62525000.0</v>
       </c>
+      <c r="D70" s="10">
+        <v>21323000.0</v>
+      </c>
+      <c r="E70" s="10">
+        <v>41202000.0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="16">
@@ -6942,6 +8092,12 @@
       <c r="C71" s="10">
         <v>0.0</v>
       </c>
+      <c r="D71" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E71" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="16">
@@ -6953,6 +8109,12 @@
       <c r="C72" s="10">
         <v>31379500.0</v>
       </c>
+      <c r="D72" s="10">
+        <v>28779500.0</v>
+      </c>
+      <c r="E72" s="10">
+        <v>2600000.0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="16">
@@ -6964,6 +8126,12 @@
       <c r="C73" s="10">
         <v>31630300.0</v>
       </c>
+      <c r="D73" s="10">
+        <v>29189300.0</v>
+      </c>
+      <c r="E73" s="10">
+        <v>2441000.0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="16">
@@ -6975,6 +8143,12 @@
       <c r="C74" s="10">
         <v>23645000.0</v>
       </c>
+      <c r="D74" s="10">
+        <v>20325000.0</v>
+      </c>
+      <c r="E74" s="10">
+        <v>3320000.0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="16">
@@ -6986,6 +8160,12 @@
       <c r="C75" s="10">
         <v>29409500.0</v>
       </c>
+      <c r="D75" s="10">
+        <v>27171500.0</v>
+      </c>
+      <c r="E75" s="10">
+        <v>2238000.0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="16">
@@ -6997,6 +8177,12 @@
       <c r="C76" s="10">
         <v>41260300.0</v>
       </c>
+      <c r="D76" s="10">
+        <v>36846300.0</v>
+      </c>
+      <c r="E76" s="10">
+        <v>4414000.0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="16">
@@ -7008,6 +8194,12 @@
       <c r="C77" s="10">
         <v>132539500.0</v>
       </c>
+      <c r="D77" s="10">
+        <v>22264500.0</v>
+      </c>
+      <c r="E77" s="10">
+        <v>110275000.0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="16">
@@ -7019,6 +8211,12 @@
       <c r="C78" s="10">
         <v>34858575.0</v>
       </c>
+      <c r="D78" s="10">
+        <v>31420500.0</v>
+      </c>
+      <c r="E78" s="10">
+        <v>3438075.0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="16">
@@ -7030,6 +8228,12 @@
       <c r="C79" s="10">
         <v>30849300.0</v>
       </c>
+      <c r="D79" s="10">
+        <v>28071300.0</v>
+      </c>
+      <c r="E79" s="10">
+        <v>2778000.0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="16">
@@ -7041,6 +8245,12 @@
       <c r="C80" s="10">
         <v>24427800.0</v>
       </c>
+      <c r="D80" s="10">
+        <v>22427800.0</v>
+      </c>
+      <c r="E80" s="10">
+        <v>2000000.0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="16">
@@ -7052,6 +8262,12 @@
       <c r="C81" s="10">
         <v>25241900.0</v>
       </c>
+      <c r="D81" s="10">
+        <v>21917200.0</v>
+      </c>
+      <c r="E81" s="10">
+        <v>3324700.0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="16">
@@ -7063,6 +8279,12 @@
       <c r="C82" s="10">
         <v>38216000.0</v>
       </c>
+      <c r="D82" s="10">
+        <v>35966000.0</v>
+      </c>
+      <c r="E82" s="10">
+        <v>2250000.0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="16">
@@ -7074,6 +8296,12 @@
       <c r="C83" s="10">
         <v>61546000.0</v>
       </c>
+      <c r="D83" s="10">
+        <v>23442000.0</v>
+      </c>
+      <c r="E83" s="10">
+        <v>38104000.0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="16">
@@ -7085,6 +8313,12 @@
       <c r="C84" s="10">
         <v>0.0</v>
       </c>
+      <c r="D84" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E84" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="16">
@@ -7096,6 +8330,12 @@
       <c r="C85" s="10">
         <v>30227400.0</v>
       </c>
+      <c r="D85" s="10">
+        <v>25688400.0</v>
+      </c>
+      <c r="E85" s="10">
+        <v>4539000.0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="16">
@@ -7107,6 +8347,12 @@
       <c r="C86" s="10">
         <v>28520000.0</v>
       </c>
+      <c r="D86" s="10">
+        <v>26092000.0</v>
+      </c>
+      <c r="E86" s="10">
+        <v>2428000.0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="16">
@@ -7118,6 +8364,12 @@
       <c r="C87" s="10">
         <v>35688100.0</v>
       </c>
+      <c r="D87" s="10">
+        <v>32317100.0</v>
+      </c>
+      <c r="E87" s="10">
+        <v>3371000.0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="16">
@@ -7129,6 +8381,12 @@
       <c r="C88" s="10">
         <v>34760500.0</v>
       </c>
+      <c r="D88" s="10">
+        <v>32767000.0</v>
+      </c>
+      <c r="E88" s="10">
+        <v>1993500.0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="16">
@@ -7140,6 +8398,12 @@
       <c r="C89" s="10">
         <v>104654000.0</v>
       </c>
+      <c r="D89" s="10">
+        <v>101476000.0</v>
+      </c>
+      <c r="E89" s="10">
+        <v>3178000.0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="16">
@@ -7151,6 +8415,12 @@
       <c r="C90" s="10">
         <v>127404000.0</v>
       </c>
+      <c r="D90" s="10">
+        <v>16764000.0</v>
+      </c>
+      <c r="E90" s="10">
+        <v>110640000.0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="16">
@@ -7162,6 +8432,12 @@
       <c r="C91" s="10">
         <v>11960500.0</v>
       </c>
+      <c r="D91" s="10">
+        <v>10100500.0</v>
+      </c>
+      <c r="E91" s="10">
+        <v>1860000.0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="16">
@@ -7173,6 +8449,12 @@
       <c r="C92" s="10">
         <v>0.0</v>
       </c>
+      <c r="D92" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E92" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="16">
@@ -7184,6 +8466,12 @@
       <c r="C93" s="10">
         <v>0.0</v>
       </c>
+      <c r="D93" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E93" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="16">
@@ -7195,6 +8483,12 @@
       <c r="C94" s="10">
         <v>0.0</v>
       </c>
+      <c r="D94" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E94" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="16">
@@ -7206,6 +8500,12 @@
       <c r="C95" s="10">
         <v>0.0</v>
       </c>
+      <c r="D95" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E95" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="16">
@@ -7217,6 +8517,12 @@
       <c r="C96" s="10">
         <v>351800.0</v>
       </c>
+      <c r="D96" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E96" s="10">
+        <v>351800.0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="16">
@@ -7228,6 +8534,12 @@
       <c r="C97" s="10">
         <v>0.0</v>
       </c>
+      <c r="D97" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E97" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="16">
@@ -7239,6 +8551,12 @@
       <c r="C98" s="10">
         <v>44656000.0</v>
       </c>
+      <c r="D98" s="10">
+        <v>6296000.0</v>
+      </c>
+      <c r="E98" s="10">
+        <v>38360000.0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="16">
@@ -7250,6 +8568,12 @@
       <c r="C99" s="10">
         <v>0.0</v>
       </c>
+      <c r="D99" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E99" s="10">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="16">
@@ -7261,94 +8585,432 @@
       <c r="C100" s="10">
         <v>0.0</v>
       </c>
+      <c r="D100" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="E100" s="10">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kategori</t>
+        </is>
+      </c>
+      <c r="B103" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nilai</t>
+        </is>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kategori</t>
-        </is>
-      </c>
-      <c r="B104" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nilai</t>
-        </is>
+      <c r="A104" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Penggunaan Pangan</t>
+        </is>
+      </c>
+      <c r="B104" s="10">
+        <v>2084847831.0</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Penggunaan Pangan</t>
+          <t xml:space="preserve">Penggunaan Operasional</t>
         </is>
       </c>
       <c r="B105" s="10">
-        <v>2084847831.0</v>
+        <v>1114049710.0</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Penggunaan Operasional</t>
+          <t xml:space="preserve">Sisa Dana</t>
         </is>
       </c>
       <c r="B106" s="10">
+        <v>288268459.0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status Hari</t>
+        </is>
+      </c>
+      <c r="B109" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jumlah</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SURPLUS</t>
+        </is>
+      </c>
+      <c r="B110" s="20">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEFISIT</t>
+        </is>
+      </c>
+      <c r="B111" s="20">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AMAN / LIBUR</t>
+        </is>
+      </c>
+      <c r="B112" s="20">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minggu</t>
+        </is>
+      </c>
+      <c r="B115" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pagu</t>
+        </is>
+      </c>
+      <c r="C115" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aktual</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surplus/Defisit</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-1</t>
+        </is>
+      </c>
+      <c r="B116" s="10">
+        <v>163046000.0</v>
+      </c>
+      <c r="C116" s="10">
+        <v>143189000.0</v>
+      </c>
+      <c r="D116" s="10">
+        <v>19857000.0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-2</t>
+        </is>
+      </c>
+      <c r="B117" s="10">
+        <v>203807500.0</v>
+      </c>
+      <c r="C117" s="10">
+        <v>198880931.0</v>
+      </c>
+      <c r="D117" s="10">
+        <v>4926569.0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-3</t>
+        </is>
+      </c>
+      <c r="B118" s="10">
+        <v>203807500.0</v>
+      </c>
+      <c r="C118" s="10">
+        <v>168575292.0</v>
+      </c>
+      <c r="D118" s="10">
+        <v>35232208.0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-4</t>
+        </is>
+      </c>
+      <c r="B119" s="10">
+        <v>203807500.0</v>
+      </c>
+      <c r="C119" s="10">
+        <v>221160500.0</v>
+      </c>
+      <c r="D119" s="10">
+        <v>-17353000.0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-5</t>
+        </is>
+      </c>
+      <c r="B120" s="10">
+        <v>203957500.0</v>
+      </c>
+      <c r="C120" s="10">
+        <v>179355250.0</v>
+      </c>
+      <c r="D120" s="10">
+        <v>24602250.0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-6</t>
+        </is>
+      </c>
+      <c r="B121" s="10">
+        <v>203957500.0</v>
+      </c>
+      <c r="C121" s="10">
+        <v>221294522.0</v>
+      </c>
+      <c r="D121" s="10">
+        <v>-17337022.0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-7</t>
+        </is>
+      </c>
+      <c r="B122" s="10">
+        <v>204007500.0</v>
+      </c>
+      <c r="C122" s="10">
+        <v>156581400.0</v>
+      </c>
+      <c r="D122" s="10">
+        <v>47426100.0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-8</t>
+        </is>
+      </c>
+      <c r="B123" s="10">
+        <v>204007500.0</v>
+      </c>
+      <c r="C123" s="10">
+        <v>238868000.0</v>
+      </c>
+      <c r="D123" s="10">
+        <v>-34860500.0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-9</t>
+        </is>
+      </c>
+      <c r="B124" s="10">
+        <v>276006000.0</v>
+      </c>
+      <c r="C124" s="10">
+        <v>222632371.0</v>
+      </c>
+      <c r="D124" s="10">
+        <v>53373629.0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-10</t>
+        </is>
+      </c>
+      <c r="B125" s="10">
+        <v>276006000.0</v>
+      </c>
+      <c r="C125" s="10">
+        <v>288106200.0</v>
+      </c>
+      <c r="D125" s="10">
+        <v>-12100200.0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-11</t>
+        </is>
+      </c>
+      <c r="B126" s="10">
+        <v>276876000.0</v>
+      </c>
+      <c r="C126" s="10">
+        <v>237028100.0</v>
+      </c>
+      <c r="D126" s="10">
+        <v>39847900.0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-12</t>
+        </is>
+      </c>
+      <c r="B127" s="10">
+        <v>276876000.0</v>
+      </c>
+      <c r="C127" s="10">
+        <v>289864100.0</v>
+      </c>
+      <c r="D127" s="10">
+        <v>-12988100.0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-13</t>
+        </is>
+      </c>
+      <c r="B128" s="10">
+        <v>276876000.0</v>
+      </c>
+      <c r="C128" s="10">
+        <v>215139575.0</v>
+      </c>
+      <c r="D128" s="10">
+        <v>61736425.0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-14</t>
+        </is>
+      </c>
+      <c r="B129" s="10">
+        <v>276876000.0</v>
+      </c>
+      <c r="C129" s="10">
+        <v>361254000.0</v>
+      </c>
+      <c r="D129" s="10">
+        <v>-84378000.0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-15</t>
+        </is>
+      </c>
+      <c r="B130" s="10">
+        <v>58182000.0</v>
+      </c>
+      <c r="C130" s="10">
+        <v>12312300.0</v>
+      </c>
+      <c r="D130" s="10">
+        <v>45869700.0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mg-16</t>
+        </is>
+      </c>
+      <c r="B131" s="10">
+        <v>29091000.0</v>
+      </c>
+      <c r="C131" s="10">
+        <v>44656000.0</v>
+      </c>
+      <c r="D131" s="10">
+        <v>-15565000.0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kategori</t>
+        </is>
+      </c>
+      <c r="B134" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anggaran</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terpakai</t>
+        </is>
+      </c>
+      <c r="D134" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pangan</t>
+        </is>
+      </c>
+      <c r="B135" s="10">
+        <v>2276180000.0</v>
+      </c>
+      <c r="C135" s="10">
+        <v>2084847831.0</v>
+      </c>
+      <c r="D135" s="10">
+        <v>191332169.0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operasional</t>
+        </is>
+      </c>
+      <c r="B136" s="10">
+        <v>1210986000.0</v>
+      </c>
+      <c r="C136" s="10">
         <v>1114049710.0</v>
       </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sisa Dana</t>
-        </is>
-      </c>
-      <c r="B107" s="10">
-        <v>138289959.0</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Status Hari</t>
-        </is>
-      </c>
-      <c r="B110" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jumlah</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SURPLUS</t>
-        </is>
-      </c>
-      <c r="B111" s="20">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DEFISIT</t>
-        </is>
-      </c>
-      <c r="B112" s="20">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AMAN</t>
-        </is>
-      </c>
-      <c r="B113" s="20">
-        <v>13</v>
+      <c r="D136" s="10">
+        <v>96936290.0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>